<commit_message>
chore: regenerate blank collection template from collection_schema
Rebuilt CLKG_采集模板.xlsx via build_template.py now that the 军垦 extension
sheets live in ingest.collection_schema (single source of truth). 9 sheets:
说明 + Place/Document/Actor/Asset + 军垦_事件/口述史/诗歌 + 词表.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data_collection/CLKG_采集模板.xlsx
+++ b/data_collection/CLKG_采集模板.xlsx
@@ -1,18 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="填写说明" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Place_地点" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Document_文档" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Actor_人物" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Asset_资产" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="词表" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Place_地点" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Document_文档" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actor_人物" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset_资产" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="军垦_事件" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="军垦_口述史" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="军垦_诗歌" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="词表" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="dv_entity_type">OFFSET('词表'!$A$2,0,0,COUNTA('词表'!$A:$A)-1,1)</definedName>
@@ -621,6 +624,286 @@
 </file>
 
 <file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>SOP</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>如 战国/西汉/奠基时期</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>如 前169年/1949年</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>发起人或行动主体</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>承受人（如适用）</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>简要描述事件内容</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>具体区域或垦区名称</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>文物、概念、物质实体</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>精神内涵、象征意义等</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>政策、组织形式等</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>书名、页码、作者等</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>数据录入者</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>资料来源出处</t>
+      </text>
+    </comment>
+    <comment ref="A2" authorId="0" shapeId="0">
+      <text>
+        <t>← 金标准示例行，照着填，填完删掉本行。</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>SOP</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>章节信息</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>节信息</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>小节信息</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>口述者姓名</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>口述者身份描述</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>采访人姓名</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>事件发生时间</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>时代分期</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>事件发生地点</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>事件涉及人物</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>涉及物品</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>涉及概念</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>触发词</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <t>行动主体</t>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <t>事件类型代码</t>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <t>事件详细描述</t>
+      </text>
+    </comment>
+    <comment ref="A2" authorId="0" shapeId="0">
+      <text>
+        <t>← 金标准示例行，照着填，填完删掉本行。</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>SOP</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>校对人/记录人</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>YYYY-MM-DD</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>填 xinjiang</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>统一填 doc</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>填原始数据 id，如 poem-001</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>诗歌标题</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>诗歌作者</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>如 汉/唐/清</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>诗歌全文</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>例证/简要说明</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>诗句中提及的地名</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>古地名对应今经纬度</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>古地名对应今经纬度</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <t>填 WGS84</t>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <t>诗歌来源文献</t>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <t>正向/负向</t>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0">
+      <text>
+        <t>情感得分</t>
+      </text>
+    </comment>
+    <comment ref="R1" authorId="0" shapeId="0">
+      <text>
+        <t>豪迈雄浑/苍凉悲悼等</t>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <t>作者身份判断</t>
+      </text>
+    </comment>
+    <comment ref="A2" authorId="0" shapeId="0">
+      <text>
+        <t>← 金标准示例行，照着填，填完删掉本行。</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment8.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>SOP</author>
@@ -2908,6 +3191,579 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00880000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>时代_历史时期</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>时间_具体年份</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>发起人</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>承受人</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>事件描述</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>地点</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>物</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>文化价值</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>屯垦制度</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>source_name_来源</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>著录人</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>出处</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>战国</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr"/>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>商鞅</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>秦国军民</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>商鞅系统阐述农战思想</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>秦国</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>农战概念</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr"/>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>战国农战政策</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>《商君书·农战》</t>
+        </is>
+      </c>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>辛佳丽</t>
+        </is>
+      </c>
+      <c r="L2" s="7" t="inlineStr">
+        <is>
+          <t>《新疆兵团屯垦戍边史》</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00884400"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>章</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>节</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>小节</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>口述者</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>口述者身份</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>采访人</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>时间</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>时代</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>地点</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>人物</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>物品</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>概念</t>
+        </is>
+      </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>触发词</t>
+        </is>
+      </c>
+      <c r="N1" s="6" t="inlineStr">
+        <is>
+          <t>行动主体</t>
+        </is>
+      </c>
+      <c r="O1" s="6" t="inlineStr">
+        <is>
+          <t>事件类型</t>
+        </is>
+      </c>
+      <c r="P1" s="5" t="inlineStr">
+        <is>
+          <t>事件描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>奠基(1949-1954)</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>向西开拔</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>（一）</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>刘双全</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>司令员</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>李霞等</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>1949年下半年</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>奠基时期</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>青海；西宁</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr"/>
+      <c r="K2" s="7" t="inlineStr"/>
+      <c r="L2" s="7" t="inlineStr"/>
+      <c r="M2" s="7" t="inlineStr">
+        <is>
+          <t>绕道青海</t>
+        </is>
+      </c>
+      <c r="N2" s="7" t="inlineStr">
+        <is>
+          <t>部队</t>
+        </is>
+      </c>
+      <c r="O2" s="7" t="inlineStr">
+        <is>
+          <t>MigrationEvent</t>
+        </is>
+      </c>
+      <c r="P2" s="7" t="inlineStr">
+        <is>
+          <t>部队从青海西宁绕道前进</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00886600"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>记录人*</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>采集日期*</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>region*</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>entity_type*</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>natural_key*</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>hasTitle_题名*</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>hasAuthor_作者</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>hasEra_时代</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>hasFullText_正文</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>hasAbstract_例证</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>hasPlace_地名</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>lon_经度</t>
+        </is>
+      </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>lat_纬度</t>
+        </is>
+      </c>
+      <c r="N1" s="6" t="inlineStr">
+        <is>
+          <t>CRS_坐标系</t>
+        </is>
+      </c>
+      <c r="O1" s="6" t="inlineStr">
+        <is>
+          <t>hasReference_出处</t>
+        </is>
+      </c>
+      <c r="P1" s="6" t="inlineStr">
+        <is>
+          <t>hasEmotion_情感极性</t>
+        </is>
+      </c>
+      <c r="Q1" s="6" t="inlineStr">
+        <is>
+          <t>hasEmotionScore_极性得分</t>
+        </is>
+      </c>
+      <c r="R1" s="6" t="inlineStr">
+        <is>
+          <t>hasEmotionType_情绪类别</t>
+        </is>
+      </c>
+      <c r="S1" s="6" t="inlineStr">
+        <is>
+          <t>hasIdentity_身份</t>
+        </is>
+      </c>
+      <c r="T1" s="6" t="inlineStr">
+        <is>
+          <t>hasNotes_备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>陈东豪</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>xinjiang</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>doc</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>poem-001</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>西极天马歌</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>刘彻</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>汉</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>天马徕兮从西极...</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>汉武虽通西域，本人未至</t>
+        </is>
+      </c>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>西极</t>
+        </is>
+      </c>
+      <c r="L2" s="7" t="inlineStr"/>
+      <c r="M2" s="7" t="inlineStr"/>
+      <c r="N2" s="7" t="inlineStr"/>
+      <c r="O2" s="7" t="inlineStr">
+        <is>
+          <t>《全汉三国晋南北朝诗》</t>
+        </is>
+      </c>
+      <c r="P2" s="7" t="inlineStr">
+        <is>
+          <t>正向</t>
+        </is>
+      </c>
+      <c r="Q2" s="7" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="R2" s="7" t="inlineStr">
+        <is>
+          <t>豪迈雄浑</t>
+        </is>
+      </c>
+      <c r="S2" s="7" t="inlineStr">
+        <is>
+          <t>想象</t>
+        </is>
+      </c>
+      <c r="T2" s="7" t="inlineStr">
+        <is>
+          <t>汉武虽通西域，本人未至</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>dv_region</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>dv_entity_type</formula1>
+    </dataValidation>
+    <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>dv_CRS</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00548235"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>

</xml_diff>